<commit_message>
feat: implement AI Agent operational logs page and resolve Next.js/Turbopack ESM build issues
</commit_message>
<xml_diff>
--- a/amc_budgetaryplan.xlsx
+++ b/amc_budgetaryplan.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="10700"/>
+    <workbookView windowWidth="25600" windowHeight="10700" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="56">
+  <si>
+    <t>N.A.</t>
+  </si>
   <si>
     <t>成本计算</t>
   </si>
@@ -35,30 +39,39 @@
     <t>套餐</t>
   </si>
   <si>
-    <t>Basic</t>
-  </si>
-  <si>
-    <t>Essential</t>
-  </si>
-  <si>
-    <t>Advanced</t>
+    <t>tier 1</t>
+  </si>
+  <si>
+    <t>tier 1 Discount</t>
+  </si>
+  <si>
+    <t>Tier 2</t>
+  </si>
+  <si>
+    <t>Tier 2 Discount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tier 2 </t>
   </si>
   <si>
     <t>品牌主理人</t>
   </si>
   <si>
-    <t>高级品牌主理人</t>
-  </si>
-  <si>
-    <t>管理预算，培训，Research 预算</t>
-  </si>
-  <si>
-    <t>Partner</t>
+    <t>资深品牌主理人</t>
+  </si>
+  <si>
+    <t>Research</t>
   </si>
   <si>
     <t>AI</t>
   </si>
   <si>
+    <t>品牌运营基本收入</t>
+  </si>
+  <si>
+    <t>培训，QA支出</t>
+  </si>
+  <si>
     <t>管理支出（管理和培训，Research)</t>
   </si>
   <si>
@@ -71,6 +84,9 @@
     <t>激励支出（品牌主理人和达人）</t>
   </si>
   <si>
+    <t>素材成本</t>
+  </si>
+  <si>
     <t>续约佣金/内部佣金</t>
   </si>
   <si>
@@ -80,12 +96,6 @@
     <t>Upsell佣金</t>
   </si>
   <si>
-    <t>销售分成 (Partner级别和公司55分，主理人和高级主理人3/7分）</t>
-  </si>
-  <si>
-    <t>分成收入</t>
-  </si>
-  <si>
     <t>第一年月利润</t>
   </si>
   <si>
@@ -105,6 +115,87 @@
   </si>
   <si>
     <t>Upsell产品佣金比例</t>
+  </si>
+  <si>
+    <t>销售佣金</t>
+  </si>
+  <si>
+    <t>基本工资</t>
+  </si>
+  <si>
+    <t>基本要求（Basic Salary*12)</t>
+  </si>
+  <si>
+    <t>奖励阶梯</t>
+  </si>
+  <si>
+    <t>计算方式</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>平台合作（外卖，团购）</t>
+  </si>
+  <si>
+    <t>上个月上线店铺的销售额</t>
+  </si>
+  <si>
+    <t>上线店铺年终总结考评跟大盘计算，走大盘奖金池</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>代运营业务（AMC10%，广告10%，点评（10%混）;</t>
+  </si>
+  <si>
+    <t>相当于卖掉10个</t>
+  </si>
+  <si>
+    <t>没有佣金，给予警告，连续三个月fail</t>
+  </si>
+  <si>
+    <t>没满足基本销售额要求</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>其他业务：自营业务3%，AI POS10%，充电宝(固定金额佣金），佣金计算向下取整）</t>
+  </si>
+  <si>
+    <t>50%佣金</t>
+  </si>
+  <si>
+    <t>满足基本营业额要求，计算50%佣金；已成为产品客户Upsell增值服务；非销售岗销售结果按照这个算；</t>
+  </si>
+  <si>
+    <t>100%佣金</t>
+  </si>
+  <si>
+    <t>超出基本要求的销售金额的销售部分</t>
+  </si>
+  <si>
+    <t>150%佣金</t>
+  </si>
+  <si>
+    <t>超出基本要求3倍的</t>
+  </si>
+  <si>
+    <t>阶梯计划</t>
+  </si>
+  <si>
+    <t>月度考核</t>
+  </si>
+  <si>
+    <t>半年度考核</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>非销售岗</t>
   </si>
 </sst>
 </file>
@@ -117,8 +208,16 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="20">
-    <font>
+  <fonts count="21">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -270,12 +369,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -590,55 +695,52 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -653,81 +755,114 @@
     <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="3" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1255,345 +1390,553 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="D6:M26"/>
+  <dimension ref="D4:O27"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="4" max="4" width="28.1875" customWidth="1"/>
-    <col min="5" max="5" width="12.6875"/>
-    <col min="6" max="6" width="9.8984375" customWidth="1"/>
-    <col min="7" max="7" width="12.6875"/>
-    <col min="10" max="10" width="10.421875" customWidth="1"/>
-    <col min="11" max="11" width="13.8046875" customWidth="1"/>
-    <col min="12" max="12" width="17.0546875" customWidth="1"/>
-    <col min="13" max="13" width="14.84375" customWidth="1"/>
+    <col min="5" max="5" width="12.6875" style="6"/>
+    <col min="6" max="6" width="12.6875" style="7"/>
+    <col min="7" max="7" width="9.8984375" style="6" customWidth="1"/>
+    <col min="8" max="8" width="12.6875" style="7"/>
+    <col min="9" max="9" width="9" style="7"/>
+    <col min="10" max="10" width="16.0625" style="6" customWidth="1"/>
+    <col min="11" max="11" width="10.421875" customWidth="1"/>
+    <col min="12" max="12" width="13.8046875" customWidth="1"/>
+    <col min="13" max="13" width="17.0546875" customWidth="1"/>
+    <col min="14" max="14" width="14.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="6" spans="4:13">
+    <row r="4" spans="4:15">
+      <c r="H4" s="7" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="4:15">
       <c r="D6" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="E6" s="6">
         <v>30</v>
       </c>
-      <c r="F6">
-        <v>30</v>
-      </c>
-      <c r="G6">
+      <c r="F6" s="7">
+        <v>50</v>
+      </c>
+      <c r="G6" s="6">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="4:13">
+      <c r="H6" s="7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="4:15">
       <c r="D7" t="s">
-        <v>1</v>
-      </c>
-      <c r="E7" t="s">
         <v>2</v>
       </c>
-      <c r="F7" t="s">
+      <c r="E7" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="G7" t="s">
+      <c r="F7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J7" t="s">
+      <c r="G7" s="8" t="s">
         <v>5</v>
       </c>
+      <c r="H7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>7</v>
+      </c>
       <c r="K7" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="4:15">
+      <c r="E8" s="6">
+        <v>800</v>
+      </c>
+      <c r="F8" s="7">
+        <v>400</v>
+      </c>
+      <c r="G8" s="6">
+        <v>3600</v>
+      </c>
+      <c r="H8" s="7">
+        <v>3600</v>
+      </c>
+      <c r="I8" s="7">
+        <v>3600</v>
+      </c>
+      <c r="O8">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="9" spans="4:15">
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="6">
+        <v>50</v>
+      </c>
+      <c r="F9" s="7">
+        <v>50</v>
+      </c>
+      <c r="G9" s="6">
+        <v>150</v>
+      </c>
+      <c r="H9" s="7">
+        <v>150</v>
+      </c>
+      <c r="I9" s="7">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="10" spans="4:15">
+      <c r="D10" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="4:13">
-      <c r="E8">
-        <v>600</v>
-      </c>
-      <c r="F8">
-        <v>1600</v>
-      </c>
-      <c r="G8">
-        <v>2600</v>
-      </c>
-    </row>
-    <row r="9" spans="4:13">
-      <c r="D9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9">
-        <v>80</v>
-      </c>
-      <c r="F9">
-        <v>120</v>
-      </c>
-      <c r="G9">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="10" spans="4:13">
-      <c r="D10" t="s">
-        <v>5</v>
-      </c>
-      <c r="E10">
-        <v>40</v>
-      </c>
-      <c r="F10">
+      <c r="E10" s="6">
         <v>60</v>
       </c>
-      <c r="G10">
-        <v>120</v>
-      </c>
-      <c r="J10">
-        <f>E10*E6</f>
+      <c r="F10" s="7">
+        <v>60</v>
+      </c>
+      <c r="G10" s="6">
+        <v>500</v>
+      </c>
+      <c r="H10" s="7">
         <v>1200</v>
+      </c>
+      <c r="I10" s="7">
+        <v>2000</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>12</v>
       </c>
       <c r="K10">
         <f>F10*F6</f>
+        <v>3000</v>
+      </c>
+      <c r="L10">
+        <f>H10*H6</f>
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="11" spans="4:15">
+      <c r="D11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="6">
+        <v>20</v>
+      </c>
+      <c r="F11" s="7">
+        <v>20</v>
+      </c>
+      <c r="G11" s="6"/>
+      <c r="L11">
+        <f>F11*F6*3</f>
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="12" spans="4:15">
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="6">
+        <v>50</v>
+      </c>
+      <c r="F12" s="7">
+        <v>50</v>
+      </c>
+      <c r="G12" s="6">
+        <v>50</v>
+      </c>
+      <c r="H12" s="7">
+        <v>50</v>
+      </c>
+      <c r="I12" s="7">
+        <v>50</v>
+      </c>
+      <c r="M12">
+        <f>E12*E6*50</f>
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="13" spans="4:15">
+      <c r="D13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="6">
+        <f>E8*10%</f>
+        <v>80</v>
+      </c>
+      <c r="F13" s="7">
+        <f>F8*10%</f>
+        <v>40</v>
+      </c>
+      <c r="G13" s="6">
+        <v>200</v>
+      </c>
+      <c r="H13" s="7">
+        <v>200</v>
+      </c>
+      <c r="I13" s="7">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="14" spans="4:15">
+      <c r="D14" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14" s="6">
+        <v>0</v>
+      </c>
+      <c r="F14" s="7">
+        <v>0</v>
+      </c>
+      <c r="G14" s="6">
+        <v>500</v>
+      </c>
+      <c r="H14" s="7">
+        <v>500</v>
+      </c>
+      <c r="I14" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="4:15">
+      <c r="D15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="6">
+        <f>E8*5%</f>
+        <v>40</v>
+      </c>
+      <c r="F15" s="7">
+        <f>F8*5%</f>
+        <v>20</v>
+      </c>
+      <c r="G15" s="6">
+        <v>150</v>
+      </c>
+      <c r="H15" s="7">
+        <v>150</v>
+      </c>
+      <c r="I15" s="7"/>
+      <c r="K15">
+        <f>F6*F15</f>
+        <v>1000</v>
+      </c>
+      <c r="L15">
+        <f>H15*H6</f>
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="16" spans="4:15">
+      <c r="D16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="4:12">
+      <c r="D18" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" s="9">
+        <v>0.05</v>
+      </c>
+      <c r="F18" s="10">
+        <v>0.05</v>
+      </c>
+      <c r="G18" s="9">
+        <v>0.05</v>
+      </c>
+      <c r="H18" s="10">
+        <v>0.05</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K18">
+        <f>E8*E18*E6</f>
+        <v>1200</v>
+      </c>
+      <c r="L18">
+        <f>H6*H8*H18</f>
         <v>1800</v>
       </c>
-      <c r="M10">
-        <f>G10*G6</f>
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="11" spans="4:13">
-      <c r="D11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E11">
-        <f>E10*30%</f>
-        <v>12</v>
-      </c>
-      <c r="F11">
-        <f>F10*30%</f>
-        <v>18</v>
-      </c>
-      <c r="G11">
-        <f>G10*30%</f>
+    </row>
+    <row r="19" spans="4:12">
+      <c r="D19" t="s">
+        <v>21</v>
+      </c>
+      <c r="E19" s="9">
+        <v>0.05</v>
+      </c>
+      <c r="F19" s="10">
+        <v>0.05</v>
+      </c>
+      <c r="G19" s="9">
+        <v>0.05</v>
+      </c>
+      <c r="H19" s="10">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="21" spans="4:12">
+      <c r="D21" t="s">
+        <v>22</v>
+      </c>
+      <c r="E21" s="6">
+        <f>E8-SUM(E9:E15)</f>
+        <v>500</v>
+      </c>
+      <c r="F21" s="7">
+        <f>F8-SUM(F9:F15)</f>
+        <v>160</v>
+      </c>
+      <c r="G21" s="6">
+        <f>G8-SUM(G9:G15)</f>
+        <v>2050</v>
+      </c>
+      <c r="H21" s="7">
+        <f>H8-SUM(H9:H15)</f>
+        <v>1350</v>
+      </c>
+      <c r="I21" s="7">
+        <f>I8-I9-I10-I13-I12-I15</f>
+        <v>1100</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="K21">
+        <f>K10+K15</f>
+        <v>4000</v>
+      </c>
+      <c r="L21">
+        <f>L10+L11+L15</f>
+        <v>16500</v>
+      </c>
+    </row>
+    <row r="22" spans="4:12">
+      <c r="D22" t="s">
+        <v>24</v>
+      </c>
+      <c r="E22" s="11">
+        <f>E21/E8</f>
+        <v>0.625</v>
+      </c>
+      <c r="F22" s="12">
+        <f>F21/F8</f>
+        <v>0.4</v>
+      </c>
+      <c r="G22" s="11">
+        <f>G21/G8</f>
+        <v>0.569444444444444</v>
+      </c>
+      <c r="H22" s="12">
+        <f>H21/H8</f>
+        <v>0.375</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="K22">
+        <f>K18+K21</f>
+        <v>5200</v>
+      </c>
+      <c r="L22">
+        <f>L18+L21</f>
+        <v>18300</v>
+      </c>
+    </row>
+    <row r="24" spans="4:12">
+      <c r="D24" t="s">
+        <v>26</v>
+      </c>
+      <c r="E24" s="6">
+        <f>E21-E8*10%+E13</f>
+        <v>500</v>
+      </c>
+      <c r="F24" s="7">
+        <f>F21-F8*10%+F13</f>
+        <v>160</v>
+      </c>
+      <c r="G24" s="6">
+        <f>G21-G8*10%+G13</f>
+        <v>1890</v>
+      </c>
+      <c r="H24" s="7">
+        <f>H21-H8*10%+H13</f>
+        <v>1190</v>
+      </c>
+    </row>
+    <row r="25" spans="4:12">
+      <c r="D25" t="s">
+        <v>27</v>
+      </c>
+      <c r="E25" s="11">
+        <f>E24/E8</f>
+        <v>0.625</v>
+      </c>
+      <c r="F25" s="12">
+        <f>F24/F8</f>
+        <v>0.4</v>
+      </c>
+      <c r="G25" s="11">
+        <f>G24/G8</f>
+        <v>0.525</v>
+      </c>
+      <c r="H25" s="12">
+        <f>H24/H8</f>
+        <v>0.330555555555556</v>
+      </c>
+    </row>
+    <row r="27" spans="4:12">
+      <c r="D27" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="B4:F15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="5"/>
+  <cols>
+    <col min="3" max="3" width="23.4375" customWidth="1"/>
+    <col min="4" max="4" width="22.6484375" customWidth="1"/>
+    <col min="5" max="5" width="49.3515625" customWidth="1"/>
+    <col min="6" max="6" width="56.109375" customWidth="1"/>
+    <col min="7" max="7" width="30.078125" customWidth="1"/>
+    <col min="8" max="8" width="14.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:6">
+      <c r="C4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6">
+      <c r="C6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6">
+      <c r="C7">
+        <v>3000</v>
+      </c>
+      <c r="D7" s="2">
+        <f>C7*12</f>
+        <v>36000</v>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1" spans="2:6">
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" t="s">
         <v>36</v>
       </c>
-      <c r="L11">
-        <f>E11*E6*50</f>
+      <c r="E8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" ht="39" customHeight="1" spans="2:6">
+      <c r="B9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" ht="68" spans="2:6">
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6">
+      <c r="E11" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6">
+      <c r="E12" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6">
+      <c r="C13" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13" t="s">
+        <v>52</v>
+      </c>
+      <c r="E13" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6">
+      <c r="C14" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14">
+        <v>36000</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6">
+      <c r="C15" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15">
         <v>18000</v>
-      </c>
-    </row>
-    <row r="12" spans="4:13">
-      <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12">
-        <v>100</v>
-      </c>
-      <c r="F12">
-        <v>200</v>
-      </c>
-      <c r="G12">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="13" spans="4:13">
-      <c r="D13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13">
-        <v>150</v>
-      </c>
-      <c r="F13">
-        <v>600</v>
-      </c>
-      <c r="G13">
-        <v>900</v>
-      </c>
-      <c r="M13">
-        <f>50*200</f>
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="14" spans="4:13">
-      <c r="D14" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14">
-        <f>E8*5%</f>
-        <v>30</v>
-      </c>
-      <c r="F14">
-        <f>F8*5%</f>
-        <v>80</v>
-      </c>
-      <c r="G14">
-        <f>G8*5%</f>
-        <v>130</v>
-      </c>
-      <c r="J14">
-        <f>E14*1/4*E6</f>
-        <v>225</v>
-      </c>
-      <c r="K14">
-        <f>F14*1/4*F6</f>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="16" spans="4:13">
-      <c r="D16" t="s">
-        <v>14</v>
-      </c>
-      <c r="E16" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="F16" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="G16" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="I16" t="s">
-        <v>15</v>
-      </c>
-      <c r="J16">
-        <f>E8*E16*E6</f>
-        <v>900</v>
-      </c>
-      <c r="K16">
-        <f>F8*F16*F6</f>
-        <v>2400</v>
-      </c>
-    </row>
-    <row r="17" spans="4:13">
-      <c r="D17" t="s">
-        <v>16</v>
-      </c>
-      <c r="E17" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="F17" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="G17" s="1">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="18" spans="4:13">
-      <c r="D18" t="s">
-        <v>17</v>
-      </c>
-      <c r="E18" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="F18" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="G18" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="I18" t="s">
-        <v>18</v>
-      </c>
-      <c r="M18">
-        <f>4000*3</f>
-        <v>12000</v>
-      </c>
-    </row>
-    <row r="20" spans="4:13">
-      <c r="D20" t="s">
-        <v>19</v>
-      </c>
-      <c r="E20">
-        <f>E8-SUM(E9:E14)</f>
-        <v>188</v>
-      </c>
-      <c r="F20">
-        <f>F8-SUM(F9:F14)</f>
-        <v>522</v>
-      </c>
-      <c r="G20">
-        <f>G8-SUM(G9:G14)</f>
-        <v>954</v>
-      </c>
-      <c r="I20" t="s">
-        <v>20</v>
-      </c>
-      <c r="J20">
-        <f>J10+J14</f>
-        <v>1425</v>
-      </c>
-      <c r="K20">
-        <f>K10+K14</f>
-        <v>2400</v>
-      </c>
-    </row>
-    <row r="21" spans="4:13">
-      <c r="D21" t="s">
-        <v>21</v>
-      </c>
-      <c r="E21" s="2">
-        <f>E20/E8</f>
-        <v>0.313333333333333</v>
-      </c>
-      <c r="F21" s="2">
-        <f>F20/F8</f>
-        <v>0.32625</v>
-      </c>
-      <c r="G21" s="2">
-        <f>G20/G8</f>
-        <v>0.366923076923077</v>
-      </c>
-      <c r="I21" t="s">
-        <v>22</v>
-      </c>
-      <c r="J21">
-        <f>J16+J20</f>
-        <v>2325</v>
-      </c>
-      <c r="K21">
-        <f>K16+K20</f>
-        <v>4800</v>
-      </c>
-      <c r="M21">
-        <f>SUM(M9:M20)</f>
-        <v>23200</v>
-      </c>
-    </row>
-    <row r="23" spans="4:13">
-      <c r="D23" t="s">
-        <v>23</v>
-      </c>
-      <c r="E23">
-        <f>E20-E8*10%+E12</f>
-        <v>228</v>
-      </c>
-      <c r="F23">
-        <f>F20-F8*10%+F12</f>
-        <v>562</v>
-      </c>
-      <c r="G23">
-        <f>G20-G8*10%+G12</f>
-        <v>994</v>
-      </c>
-    </row>
-    <row r="24" spans="4:13">
-      <c r="D24" t="s">
-        <v>24</v>
-      </c>
-      <c r="E24" s="2">
-        <f>E23/E8</f>
-        <v>0.38</v>
-      </c>
-      <c r="F24" s="2">
-        <f>F23/F8</f>
-        <v>0.35125</v>
-      </c>
-      <c r="G24" s="2">
-        <f>G23/G8</f>
-        <v>0.382307692307692</v>
-      </c>
-    </row>
-    <row r="26" spans="4:13">
-      <c r="D26" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(companion): support TRIGGER_UPLOAD voice intent to open photo library
</commit_message>
<xml_diff>
--- a/amc_budgetaryplan.xlsx
+++ b/amc_budgetaryplan.xlsx
@@ -135,6 +135,21 @@
     <t>A</t>
   </si>
   <si>
+    <t>代运营业务（AMC10%，点评（10%混）;</t>
+  </si>
+  <si>
+    <t>相当于卖掉10个</t>
+  </si>
+  <si>
+    <t>没有佣金，给予警告，连续三个月fail</t>
+  </si>
+  <si>
+    <t>没满足基本销售额要求</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
     <t>平台合作（外卖，团购）</t>
   </si>
   <si>
@@ -142,21 +157,6 @@
   </si>
   <si>
     <t>上线店铺年终总结考评跟大盘计算，走大盘奖金池</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>代运营业务（AMC10%，广告10%，点评（10%混）;</t>
-  </si>
-  <si>
-    <t>相当于卖掉10个</t>
-  </si>
-  <si>
-    <t>没有佣金，给予警告，连续三个月fail</t>
-  </si>
-  <si>
-    <t>没满足基本销售额要求</t>
   </si>
   <si>
     <t>C</t>
@@ -825,7 +825,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -833,6 +833,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -841,22 +850,10 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1">
@@ -1394,12 +1391,12 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="4" max="4" width="28.1875" customWidth="1"/>
-    <col min="5" max="5" width="12.6875" style="6"/>
-    <col min="6" max="6" width="12.6875" style="7"/>
-    <col min="7" max="7" width="9.8984375" style="6" customWidth="1"/>
-    <col min="8" max="8" width="12.6875" style="7"/>
-    <col min="9" max="9" width="9" style="7"/>
-    <col min="10" max="10" width="16.0625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="12.6875" style="8"/>
+    <col min="6" max="6" width="12.6875" style="3"/>
+    <col min="7" max="7" width="9.8984375" style="8" customWidth="1"/>
+    <col min="8" max="8" width="12.6875" style="3"/>
+    <col min="9" max="9" width="9" style="3"/>
+    <col min="10" max="10" width="16.0625" style="8" customWidth="1"/>
     <col min="11" max="11" width="10.421875" customWidth="1"/>
     <col min="12" max="12" width="13.8046875" customWidth="1"/>
     <col min="13" max="13" width="17.0546875" customWidth="1"/>
@@ -1407,7 +1404,7 @@
   </cols>
   <sheetData>
     <row r="4" spans="4:15">
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="3" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1415,16 +1412,16 @@
       <c r="D6" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="8">
         <v>30</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="3">
         <v>50</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="8">
         <v>10</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="3">
         <v>10</v>
       </c>
     </row>
@@ -1435,16 +1432,16 @@
       <c r="E7" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="I7" s="3" t="s">
         <v>7</v>
       </c>
       <c r="K7" t="s">
@@ -1458,19 +1455,19 @@
       </c>
     </row>
     <row r="8" spans="4:15">
-      <c r="E8" s="6">
+      <c r="E8" s="8">
         <v>800</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="3">
         <v>400</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="8">
         <v>3600</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="3">
         <v>3600</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="3">
         <v>3600</v>
       </c>
       <c r="O8">
@@ -1481,19 +1478,19 @@
       <c r="D9" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="8">
         <v>50</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="3">
         <v>50</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="8">
         <v>150</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="3">
         <v>150</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="3">
         <v>150</v>
       </c>
     </row>
@@ -1501,19 +1498,19 @@
       <c r="D10" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="8">
         <v>60</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="3">
         <v>60</v>
       </c>
-      <c r="G10" s="6">
+      <c r="G10" s="8">
         <v>500</v>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="3">
         <v>1200</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="3">
         <v>2000</v>
       </c>
       <c r="J10" s="8" t="s">
@@ -1532,13 +1529,12 @@
       <c r="D11" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="8">
         <v>20</v>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="3">
         <v>20</v>
       </c>
-      <c r="G11" s="6"/>
       <c r="L11">
         <f>F11*F6*3</f>
         <v>3000</v>
@@ -1548,19 +1544,19 @@
       <c r="D12" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="8">
         <v>50</v>
       </c>
-      <c r="F12" s="7">
+      <c r="F12" s="3">
         <v>50</v>
       </c>
-      <c r="G12" s="6">
+      <c r="G12" s="8">
         <v>50</v>
       </c>
-      <c r="H12" s="7">
+      <c r="H12" s="3">
         <v>50</v>
       </c>
-      <c r="I12" s="7">
+      <c r="I12" s="3">
         <v>50</v>
       </c>
       <c r="M12">
@@ -1572,21 +1568,21 @@
       <c r="D13" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="8">
         <f>E8*10%</f>
         <v>80</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13" s="3">
         <f>F8*10%</f>
         <v>40</v>
       </c>
-      <c r="G13" s="6">
+      <c r="G13" s="8">
         <v>200</v>
       </c>
-      <c r="H13" s="7">
+      <c r="H13" s="3">
         <v>200</v>
       </c>
-      <c r="I13" s="7">
+      <c r="I13" s="3">
         <v>300</v>
       </c>
     </row>
@@ -1594,19 +1590,19 @@
       <c r="D14" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="8">
         <v>0</v>
       </c>
-      <c r="F14" s="7">
+      <c r="F14" s="3">
         <v>0</v>
       </c>
-      <c r="G14" s="6">
+      <c r="G14" s="8">
         <v>500</v>
       </c>
-      <c r="H14" s="7">
+      <c r="H14" s="3">
         <v>500</v>
       </c>
-      <c r="I14" s="7">
+      <c r="I14" s="3">
         <v>0</v>
       </c>
     </row>
@@ -1614,21 +1610,20 @@
       <c r="D15" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="8">
         <f>E8*5%</f>
         <v>40</v>
       </c>
-      <c r="F15" s="7">
+      <c r="F15" s="3">
         <f>F8*5%</f>
         <v>20</v>
       </c>
-      <c r="G15" s="6">
+      <c r="G15" s="8">
         <v>150</v>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="3">
         <v>150</v>
       </c>
-      <c r="I15" s="7"/>
       <c r="K15">
         <f>F6*F15</f>
         <v>1000</v>
@@ -1650,13 +1645,13 @@
       <c r="E18" s="9">
         <v>0.05</v>
       </c>
-      <c r="F18" s="10">
+      <c r="F18" s="7">
         <v>0.05</v>
       </c>
       <c r="G18" s="9">
         <v>0.05</v>
       </c>
-      <c r="H18" s="10">
+      <c r="H18" s="7">
         <v>0.05</v>
       </c>
       <c r="J18" s="8" t="s">
@@ -1678,13 +1673,13 @@
       <c r="E19" s="9">
         <v>0.05</v>
       </c>
-      <c r="F19" s="10">
+      <c r="F19" s="7">
         <v>0.05</v>
       </c>
       <c r="G19" s="9">
         <v>0.05</v>
       </c>
-      <c r="H19" s="10">
+      <c r="H19" s="7">
         <v>0.05</v>
       </c>
     </row>
@@ -1692,23 +1687,23 @@
       <c r="D21" t="s">
         <v>22</v>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="8">
         <f>E8-SUM(E9:E15)</f>
         <v>500</v>
       </c>
-      <c r="F21" s="7">
+      <c r="F21" s="3">
         <f>F8-SUM(F9:F15)</f>
         <v>160</v>
       </c>
-      <c r="G21" s="6">
+      <c r="G21" s="8">
         <f>G8-SUM(G9:G15)</f>
         <v>2050</v>
       </c>
-      <c r="H21" s="7">
+      <c r="H21" s="3">
         <f>H8-SUM(H9:H15)</f>
         <v>1350</v>
       </c>
-      <c r="I21" s="7">
+      <c r="I21" s="3">
         <f>I8-I9-I10-I13-I12-I15</f>
         <v>1100</v>
       </c>
@@ -1728,19 +1723,19 @@
       <c r="D22" t="s">
         <v>24</v>
       </c>
-      <c r="E22" s="11">
+      <c r="E22" s="10">
         <f>E21/E8</f>
         <v>0.625</v>
       </c>
-      <c r="F22" s="12">
+      <c r="F22" s="11">
         <f>F21/F8</f>
         <v>0.4</v>
       </c>
-      <c r="G22" s="11">
+      <c r="G22" s="10">
         <f>G21/G8</f>
         <v>0.569444444444444</v>
       </c>
-      <c r="H22" s="12">
+      <c r="H22" s="11">
         <f>H21/H8</f>
         <v>0.375</v>
       </c>
@@ -1760,19 +1755,19 @@
       <c r="D24" t="s">
         <v>26</v>
       </c>
-      <c r="E24" s="6">
+      <c r="E24" s="8">
         <f>E21-E8*10%+E13</f>
         <v>500</v>
       </c>
-      <c r="F24" s="7">
+      <c r="F24" s="3">
         <f>F21-F8*10%+F13</f>
         <v>160</v>
       </c>
-      <c r="G24" s="6">
+      <c r="G24" s="8">
         <f>G21-G8*10%+G13</f>
         <v>1890</v>
       </c>
-      <c r="H24" s="7">
+      <c r="H24" s="3">
         <f>H21-H8*10%+H13</f>
         <v>1190</v>
       </c>
@@ -1781,19 +1776,19 @@
       <c r="D25" t="s">
         <v>27</v>
       </c>
-      <c r="E25" s="11">
+      <c r="E25" s="10">
         <f>E24/E8</f>
         <v>0.625</v>
       </c>
-      <c r="F25" s="12">
+      <c r="F25" s="11">
         <f>F24/F8</f>
         <v>0.4</v>
       </c>
-      <c r="G25" s="11">
+      <c r="G25" s="10">
         <f>G24/G8</f>
         <v>0.525</v>
       </c>
-      <c r="H25" s="12">
+      <c r="H25" s="11">
         <f>H24/H8</f>
         <v>0.330555555555556</v>
       </c>
@@ -1815,9 +1810,10 @@
   <dimension ref="B4:F15"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="5"/>
   <cols>
-    <col min="3" max="3" width="23.4375" customWidth="1"/>
-    <col min="4" max="4" width="22.6484375" customWidth="1"/>
-    <col min="5" max="5" width="49.3515625" customWidth="1"/>
+    <col min="2" max="2" width="4.9765625" customWidth="1"/>
+    <col min="3" max="3" width="24.375" customWidth="1"/>
+    <col min="4" max="4" width="24.484375" customWidth="1"/>
+    <col min="5" max="5" width="31.8125" customWidth="1"/>
     <col min="6" max="6" width="56.109375" customWidth="1"/>
     <col min="7" max="7" width="30.078125" customWidth="1"/>
     <col min="8" max="8" width="14.453125" customWidth="1"/>
@@ -1828,17 +1824,17 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="2:6">
-      <c r="C6" s="1" t="s">
+    <row r="6" s="1" customFormat="1" spans="2:6">
+      <c r="C6" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="3" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1851,64 +1847,64 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1" spans="2:6">
-      <c r="B8" t="s">
+    <row r="8" s="2" customFormat="1" ht="39" customHeight="1" spans="2:6">
+      <c r="B8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="5" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="9" ht="39" customHeight="1" spans="2:6">
+      <c r="F8" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" customFormat="1" ht="48" customHeight="1" spans="2:6">
       <c r="B9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C9" s="3" t="s">
         <v>39</v>
       </c>
+      <c r="C9" t="s">
+        <v>40</v>
+      </c>
       <c r="D9" t="s">
-        <v>40</v>
-      </c>
-      <c r="E9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="E9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="10" ht="68" spans="2:6">
+    <row r="10" ht="63" customHeight="1" spans="2:6">
       <c r="B10" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="3" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="11" spans="2:6">
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="3" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="12" spans="2:6">
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F12" s="3" t="s">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
prd(auth): refine brand auto-binding and assignment pool logic in prd
</commit_message>
<xml_diff>
--- a/amc_budgetaryplan.xlsx
+++ b/amc_budgetaryplan.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="10700" activeTab="1"/>
+    <workbookView windowHeight="10700" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -120,10 +120,10 @@
     <t>销售佣金</t>
   </si>
   <si>
-    <t>基本工资</t>
-  </si>
-  <si>
-    <t>基本要求（Basic Salary*12)</t>
+    <t>Gross Salary</t>
+  </si>
+  <si>
+    <t>基本要求（Gross Salary*12)</t>
   </si>
   <si>
     <t>奖励阶梯</t>
@@ -825,7 +825,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -833,9 +833,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1391,12 +1388,12 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="4" max="4" width="28.1875" customWidth="1"/>
-    <col min="5" max="5" width="12.6875" style="8"/>
-    <col min="6" max="6" width="12.6875" style="3"/>
-    <col min="7" max="7" width="9.8984375" style="8" customWidth="1"/>
-    <col min="8" max="8" width="12.6875" style="3"/>
-    <col min="9" max="9" width="9" style="3"/>
-    <col min="10" max="10" width="16.0625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="12.6875" style="7"/>
+    <col min="6" max="6" width="12.6875" style="1"/>
+    <col min="7" max="7" width="9.8984375" style="7" customWidth="1"/>
+    <col min="8" max="8" width="12.6875" style="1"/>
+    <col min="9" max="9" width="9" style="1"/>
+    <col min="10" max="10" width="16.0625" style="7" customWidth="1"/>
     <col min="11" max="11" width="10.421875" customWidth="1"/>
     <col min="12" max="12" width="13.8046875" customWidth="1"/>
     <col min="13" max="13" width="17.0546875" customWidth="1"/>
@@ -1404,7 +1401,7 @@
   </cols>
   <sheetData>
     <row r="4" spans="4:15">
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="1" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1412,16 +1409,16 @@
       <c r="D6" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="7">
         <v>30</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="1">
         <v>50</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="7">
         <v>10</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="1">
         <v>10</v>
       </c>
     </row>
@@ -1429,19 +1426,19 @@
       <c r="D7" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="K7" t="s">
@@ -1455,19 +1452,19 @@
       </c>
     </row>
     <row r="8" spans="4:15">
-      <c r="E8" s="8">
+      <c r="E8" s="7">
         <v>800</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="1">
         <v>400</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="7">
         <v>3600</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="1">
         <v>3600</v>
       </c>
-      <c r="I8" s="3">
+      <c r="I8" s="1">
         <v>3600</v>
       </c>
       <c r="O8">
@@ -1478,19 +1475,19 @@
       <c r="D9" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="7">
         <v>50</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="1">
         <v>50</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="7">
         <v>150</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="1">
         <v>150</v>
       </c>
-      <c r="I9" s="3">
+      <c r="I9" s="1">
         <v>150</v>
       </c>
     </row>
@@ -1498,22 +1495,22 @@
       <c r="D10" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="7">
         <v>60</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="1">
         <v>60</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="7">
         <v>500</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="1">
         <v>1200</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="1">
         <v>2000</v>
       </c>
-      <c r="J10" s="8" t="s">
+      <c r="J10" s="7" t="s">
         <v>12</v>
       </c>
       <c r="K10">
@@ -1529,10 +1526,10 @@
       <c r="D11" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="7">
         <v>20</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="1">
         <v>20</v>
       </c>
       <c r="L11">
@@ -1544,19 +1541,19 @@
       <c r="D12" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="7">
         <v>50</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="1">
         <v>50</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="7">
         <v>50</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="1">
         <v>50</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="1">
         <v>50</v>
       </c>
       <c r="M12">
@@ -1568,21 +1565,21 @@
       <c r="D13" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="7">
         <f>E8*10%</f>
         <v>80</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13" s="1">
         <f>F8*10%</f>
         <v>40</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="7">
         <v>200</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="1">
         <v>200</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="1">
         <v>300</v>
       </c>
     </row>
@@ -1590,19 +1587,19 @@
       <c r="D14" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="8">
+      <c r="E14" s="7">
         <v>0</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="1">
         <v>0</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="7">
         <v>500</v>
       </c>
-      <c r="H14" s="3">
+      <c r="H14" s="1">
         <v>500</v>
       </c>
-      <c r="I14" s="3">
+      <c r="I14" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1610,18 +1607,18 @@
       <c r="D15" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="8">
+      <c r="E15" s="7">
         <f>E8*5%</f>
         <v>40</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="1">
         <f>F8*5%</f>
         <v>20</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="7">
         <v>150</v>
       </c>
-      <c r="H15" s="3">
+      <c r="H15" s="1">
         <v>150</v>
       </c>
       <c r="K15">
@@ -1642,19 +1639,19 @@
       <c r="D18" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="8">
         <v>0.05</v>
       </c>
-      <c r="F18" s="7">
+      <c r="F18" s="6">
         <v>0.05</v>
       </c>
-      <c r="G18" s="9">
+      <c r="G18" s="8">
         <v>0.05</v>
       </c>
-      <c r="H18" s="7">
+      <c r="H18" s="6">
         <v>0.05</v>
       </c>
-      <c r="J18" s="8" t="s">
+      <c r="J18" s="7" t="s">
         <v>20</v>
       </c>
       <c r="K18">
@@ -1670,16 +1667,16 @@
       <c r="D19" t="s">
         <v>21</v>
       </c>
-      <c r="E19" s="9">
+      <c r="E19" s="8">
         <v>0.05</v>
       </c>
-      <c r="F19" s="7">
+      <c r="F19" s="6">
         <v>0.05</v>
       </c>
-      <c r="G19" s="9">
+      <c r="G19" s="8">
         <v>0.05</v>
       </c>
-      <c r="H19" s="7">
+      <c r="H19" s="6">
         <v>0.05</v>
       </c>
     </row>
@@ -1687,27 +1684,27 @@
       <c r="D21" t="s">
         <v>22</v>
       </c>
-      <c r="E21" s="8">
+      <c r="E21" s="7">
         <f>E8-SUM(E9:E15)</f>
         <v>500</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F21" s="1">
         <f>F8-SUM(F9:F15)</f>
         <v>160</v>
       </c>
-      <c r="G21" s="8">
+      <c r="G21" s="7">
         <f>G8-SUM(G9:G15)</f>
         <v>2050</v>
       </c>
-      <c r="H21" s="3">
+      <c r="H21" s="1">
         <f>H8-SUM(H9:H15)</f>
         <v>1350</v>
       </c>
-      <c r="I21" s="3">
+      <c r="I21" s="1">
         <f>I8-I9-I10-I13-I12-I15</f>
         <v>1100</v>
       </c>
-      <c r="J21" s="8" t="s">
+      <c r="J21" s="7" t="s">
         <v>23</v>
       </c>
       <c r="K21">
@@ -1723,23 +1720,23 @@
       <c r="D22" t="s">
         <v>24</v>
       </c>
-      <c r="E22" s="10">
+      <c r="E22" s="9">
         <f>E21/E8</f>
         <v>0.625</v>
       </c>
-      <c r="F22" s="11">
+      <c r="F22" s="10">
         <f>F21/F8</f>
         <v>0.4</v>
       </c>
-      <c r="G22" s="10">
+      <c r="G22" s="9">
         <f>G21/G8</f>
         <v>0.569444444444444</v>
       </c>
-      <c r="H22" s="11">
+      <c r="H22" s="10">
         <f>H21/H8</f>
         <v>0.375</v>
       </c>
-      <c r="J22" s="8" t="s">
+      <c r="J22" s="7" t="s">
         <v>25</v>
       </c>
       <c r="K22">
@@ -1755,19 +1752,19 @@
       <c r="D24" t="s">
         <v>26</v>
       </c>
-      <c r="E24" s="8">
+      <c r="E24" s="7">
         <f>E21-E8*10%+E13</f>
         <v>500</v>
       </c>
-      <c r="F24" s="3">
+      <c r="F24" s="1">
         <f>F21-F8*10%+F13</f>
         <v>160</v>
       </c>
-      <c r="G24" s="8">
+      <c r="G24" s="7">
         <f>G21-G8*10%+G13</f>
         <v>1890</v>
       </c>
-      <c r="H24" s="3">
+      <c r="H24" s="1">
         <f>H21-H8*10%+H13</f>
         <v>1190</v>
       </c>
@@ -1776,19 +1773,19 @@
       <c r="D25" t="s">
         <v>27</v>
       </c>
-      <c r="E25" s="10">
+      <c r="E25" s="9">
         <f>E24/E8</f>
         <v>0.625</v>
       </c>
-      <c r="F25" s="11">
+      <c r="F25" s="10">
         <f>F24/F8</f>
         <v>0.4</v>
       </c>
-      <c r="G25" s="10">
+      <c r="G25" s="9">
         <f>G24/G8</f>
         <v>0.525</v>
       </c>
-      <c r="H25" s="11">
+      <c r="H25" s="10">
         <f>H24/H8</f>
         <v>0.330555555555556</v>
       </c>
@@ -1825,42 +1822,42 @@
       </c>
     </row>
     <row r="6" s="1" customFormat="1" spans="2:6">
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="1" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="2:6">
       <c r="C7">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="D7" s="2">
         <f>C7*12</f>
-        <v>36000</v>
+        <v>42000</v>
       </c>
     </row>
     <row r="8" s="2" customFormat="1" ht="39" customHeight="1" spans="2:6">
       <c r="B8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>35</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="4" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1882,34 +1879,34 @@
       <c r="B10" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="11" spans="2:6">
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="1" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="12" spans="2:6">
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="13" spans="2:6">
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="4" t="s">
         <v>51</v>
       </c>
       <c r="D13" t="s">

</xml_diff>

<commit_message>
feat(auth): add Singapore PDPA privacy policy and terms of service
</commit_message>
<xml_diff>
--- a/amc_budgetaryplan.xlsx
+++ b/amc_budgetaryplan.xlsx
@@ -4,11 +4,12 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="10700" activeTab="1"/>
+    <workbookView windowHeight="10700"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="57">
   <si>
     <t>N.A.</t>
   </si>
@@ -42,7 +43,7 @@
     <t>tier 1</t>
   </si>
   <si>
-    <t>tier 1 Discount</t>
+    <t>Tier 1 Discount</t>
   </si>
   <si>
     <t>Tier 2</t>
@@ -67,6 +68,9 @@
   </si>
   <si>
     <t>品牌运营基本收入</t>
+  </si>
+  <si>
+    <t>高级品牌主理人</t>
   </si>
   <si>
     <t>培训，QA支出</t>
@@ -825,11 +829,17 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
@@ -845,6 +855,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -1384,16 +1397,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="D4:O27"/>
+  <dimension ref="D4:O28"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="4" max="4" width="28.1875" customWidth="1"/>
-    <col min="5" max="5" width="12.6875" style="7"/>
-    <col min="6" max="6" width="12.6875" style="1"/>
-    <col min="7" max="7" width="9.8984375" style="7" customWidth="1"/>
-    <col min="8" max="8" width="12.6875" style="1"/>
-    <col min="9" max="9" width="9" style="1"/>
-    <col min="10" max="10" width="16.0625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="12.6875" style="10"/>
+    <col min="6" max="6" width="14.625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="12.890625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="12.6875" style="2"/>
+    <col min="9" max="9" width="9" style="2"/>
+    <col min="10" max="10" width="16.0625" style="10" customWidth="1"/>
     <col min="11" max="11" width="10.421875" customWidth="1"/>
     <col min="12" max="12" width="13.8046875" customWidth="1"/>
     <col min="13" max="13" width="17.0546875" customWidth="1"/>
@@ -1401,7 +1414,7 @@
   </cols>
   <sheetData>
     <row r="4" spans="4:15">
-      <c r="H4" s="1" t="s">
+      <c r="H4" s="2" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1409,16 +1422,16 @@
       <c r="D6" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="10">
         <v>30</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="2">
         <v>50</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="10">
         <v>10</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>10</v>
       </c>
     </row>
@@ -1426,19 +1439,19 @@
       <c r="D7" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="I7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="K7" t="s">
@@ -1452,19 +1465,19 @@
       </c>
     </row>
     <row r="8" spans="4:15">
-      <c r="E8" s="7">
+      <c r="E8" s="10">
         <v>800</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="2">
         <v>400</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="10">
         <v>3600</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>3600</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="2">
         <v>3600</v>
       </c>
       <c r="O8">
@@ -1475,19 +1488,19 @@
       <c r="D9" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="10">
         <v>50</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9" s="2">
         <v>50</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="10">
         <v>150</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>150</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="2">
         <v>150</v>
       </c>
     </row>
@@ -1495,22 +1508,22 @@
       <c r="D10" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="10">
         <v>60</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="2">
         <v>60</v>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="10">
         <v>500</v>
       </c>
-      <c r="H10" s="1">
-        <v>1200</v>
-      </c>
-      <c r="I10" s="1">
+      <c r="H10" s="2">
+        <v>180</v>
+      </c>
+      <c r="I10" s="2">
         <v>2000</v>
       </c>
-      <c r="J10" s="7" t="s">
+      <c r="J10" s="10" t="s">
         <v>12</v>
       </c>
       <c r="K10">
@@ -1519,280 +1532,288 @@
       </c>
       <c r="L10">
         <f>H10*H6</f>
-        <v>12000</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="11" spans="4:15">
       <c r="D11" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="7">
-        <v>20</v>
-      </c>
-      <c r="F11" s="1">
-        <v>20</v>
-      </c>
-      <c r="L11">
-        <f>F11*F6*3</f>
-        <v>3000</v>
+      <c r="H11" s="2">
+        <v>1200</v>
       </c>
     </row>
     <row r="12" spans="4:15">
       <c r="D12" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="7">
-        <v>50</v>
-      </c>
-      <c r="F12" s="1">
-        <v>50</v>
-      </c>
-      <c r="G12" s="7">
-        <v>50</v>
-      </c>
-      <c r="H12" s="1">
-        <v>50</v>
-      </c>
-      <c r="I12" s="1">
-        <v>50</v>
-      </c>
-      <c r="M12">
-        <f>E12*E6*50</f>
-        <v>75000</v>
+      <c r="E12" s="10">
+        <v>20</v>
+      </c>
+      <c r="F12" s="2">
+        <v>20</v>
+      </c>
+      <c r="L12">
+        <f>F12*F6*3</f>
+        <v>3000</v>
       </c>
     </row>
     <row r="13" spans="4:15">
       <c r="D13" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="7">
-        <f>E8*10%</f>
-        <v>80</v>
-      </c>
-      <c r="F13" s="1">
-        <f>F8*10%</f>
-        <v>40</v>
-      </c>
-      <c r="G13" s="7">
-        <v>200</v>
-      </c>
-      <c r="H13" s="1">
-        <v>200</v>
-      </c>
-      <c r="I13" s="1">
-        <v>300</v>
+      <c r="E13" s="10">
+        <v>50</v>
+      </c>
+      <c r="F13" s="2">
+        <v>50</v>
+      </c>
+      <c r="G13" s="10">
+        <v>50</v>
+      </c>
+      <c r="H13" s="2">
+        <v>50</v>
+      </c>
+      <c r="I13" s="2">
+        <v>50</v>
+      </c>
+      <c r="M13">
+        <f>E13*E6*50</f>
+        <v>75000</v>
       </c>
     </row>
     <row r="14" spans="4:15">
       <c r="D14" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="7">
-        <v>0</v>
-      </c>
-      <c r="F14" s="1">
-        <v>0</v>
-      </c>
-      <c r="G14" s="7">
-        <v>500</v>
-      </c>
-      <c r="H14" s="1">
-        <v>500</v>
-      </c>
-      <c r="I14" s="1">
-        <v>0</v>
+      <c r="E14" s="10">
+        <f>E8*10%</f>
+        <v>80</v>
+      </c>
+      <c r="F14" s="2">
+        <f>F8*10%</f>
+        <v>40</v>
+      </c>
+      <c r="G14" s="10">
+        <v>200</v>
+      </c>
+      <c r="H14" s="2">
+        <v>200</v>
+      </c>
+      <c r="I14" s="2">
+        <v>300</v>
       </c>
     </row>
     <row r="15" spans="4:15">
       <c r="D15" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="7">
-        <f>E8*5%</f>
-        <v>40</v>
-      </c>
-      <c r="F15" s="1">
-        <f>F8*5%</f>
-        <v>20</v>
-      </c>
-      <c r="G15" s="7">
-        <v>150</v>
-      </c>
-      <c r="H15" s="1">
-        <v>150</v>
-      </c>
-      <c r="K15">
-        <f>F6*F15</f>
-        <v>1000</v>
-      </c>
-      <c r="L15">
-        <f>H15*H6</f>
-        <v>1500</v>
+      <c r="E15" s="10">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0</v>
+      </c>
+      <c r="G15" s="10">
+        <v>500</v>
+      </c>
+      <c r="H15" s="2">
+        <v>500</v>
+      </c>
+      <c r="I15" s="2">
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="4:15">
       <c r="D16" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="18" spans="4:12">
-      <c r="D18" t="s">
+      <c r="E16" s="10">
+        <f>E8*5%</f>
+        <v>40</v>
+      </c>
+      <c r="F16" s="2">
+        <f>F8*5%</f>
+        <v>20</v>
+      </c>
+      <c r="G16" s="10">
+        <v>150</v>
+      </c>
+      <c r="H16" s="2">
+        <v>150</v>
+      </c>
+      <c r="K16">
+        <f>F6*F16</f>
+        <v>1000</v>
+      </c>
+      <c r="L16">
+        <f>H16*H6</f>
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="17" spans="4:12">
+      <c r="D17" t="s">
         <v>19</v>
-      </c>
-      <c r="E18" s="8">
-        <v>0.05</v>
-      </c>
-      <c r="F18" s="6">
-        <v>0.05</v>
-      </c>
-      <c r="G18" s="8">
-        <v>0.05</v>
-      </c>
-      <c r="H18" s="6">
-        <v>0.05</v>
-      </c>
-      <c r="J18" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="K18">
-        <f>E8*E18*E6</f>
-        <v>1200</v>
-      </c>
-      <c r="L18">
-        <f>H6*H8*H18</f>
-        <v>1800</v>
       </c>
     </row>
     <row r="19" spans="4:12">
       <c r="D19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" s="11">
+        <v>0.05</v>
+      </c>
+      <c r="F19" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="G19" s="11">
+        <v>0.05</v>
+      </c>
+      <c r="H19" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="J19" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="E19" s="8">
+      <c r="K19">
+        <f>E8*E19*E6</f>
+        <v>1200</v>
+      </c>
+      <c r="L19">
+        <f>H6*H8*H19</f>
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="20" spans="4:12">
+      <c r="D20" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20" s="11">
         <v>0.05</v>
       </c>
-      <c r="F19" s="6">
+      <c r="F20" s="8">
         <v>0.05</v>
       </c>
-      <c r="G19" s="8">
+      <c r="G20" s="11">
         <v>0.05</v>
       </c>
-      <c r="H19" s="6">
+      <c r="H20" s="8">
         <v>0.05</v>
-      </c>
-    </row>
-    <row r="21" spans="4:12">
-      <c r="D21" t="s">
-        <v>22</v>
-      </c>
-      <c r="E21" s="7">
-        <f>E8-SUM(E9:E15)</f>
-        <v>500</v>
-      </c>
-      <c r="F21" s="1">
-        <f>F8-SUM(F9:F15)</f>
-        <v>160</v>
-      </c>
-      <c r="G21" s="7">
-        <f>G8-SUM(G9:G15)</f>
-        <v>2050</v>
-      </c>
-      <c r="H21" s="1">
-        <f>H8-SUM(H9:H15)</f>
-        <v>1350</v>
-      </c>
-      <c r="I21" s="1">
-        <f>I8-I9-I10-I13-I12-I15</f>
-        <v>1100</v>
-      </c>
-      <c r="J21" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="K21">
-        <f>K10+K15</f>
-        <v>4000</v>
-      </c>
-      <c r="L21">
-        <f>L10+L11+L15</f>
-        <v>16500</v>
       </c>
     </row>
     <row r="22" spans="4:12">
       <c r="D22" t="s">
+        <v>23</v>
+      </c>
+      <c r="E22" s="10">
+        <f>E8-SUM(E9:E16)</f>
+        <v>500</v>
+      </c>
+      <c r="F22" s="2">
+        <f>F8-SUM(F9:F16)</f>
+        <v>160</v>
+      </c>
+      <c r="G22" s="10">
+        <f>G8-SUM(G9:G16)</f>
+        <v>2050</v>
+      </c>
+      <c r="H22" s="2">
+        <f>H8-SUM(H9:H16)</f>
+        <v>1170</v>
+      </c>
+      <c r="I22" s="2">
+        <f>I8-I9-I10-I14-I13-I16</f>
+        <v>1100</v>
+      </c>
+      <c r="J22" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E22" s="9">
-        <f>E21/E8</f>
+      <c r="K22">
+        <f>K10+K16</f>
+        <v>4000</v>
+      </c>
+      <c r="L22">
+        <f>L10+L12+L16</f>
+        <v>6300</v>
+      </c>
+    </row>
+    <row r="23" spans="4:12">
+      <c r="D23" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="12">
+        <f>E22/E8</f>
         <v>0.625</v>
       </c>
-      <c r="F22" s="10">
-        <f>F21/F8</f>
+      <c r="F23" s="13">
+        <f>F22/F8</f>
         <v>0.4</v>
       </c>
-      <c r="G22" s="9">
-        <f>G21/G8</f>
+      <c r="G23" s="12">
+        <f>G22/G8</f>
         <v>0.569444444444444</v>
       </c>
-      <c r="H22" s="10">
-        <f>H21/H8</f>
-        <v>0.375</v>
-      </c>
-      <c r="J22" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="K22">
-        <f>K18+K21</f>
+      <c r="H23" s="13">
+        <f>H22/H8</f>
+        <v>0.325</v>
+      </c>
+      <c r="J23" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K23">
+        <f>K19+K22</f>
         <v>5200</v>
       </c>
-      <c r="L22">
-        <f>L18+L21</f>
-        <v>18300</v>
-      </c>
-    </row>
-    <row r="24" spans="4:12">
-      <c r="D24" t="s">
-        <v>26</v>
-      </c>
-      <c r="E24" s="7">
-        <f>E21-E8*10%+E13</f>
-        <v>500</v>
-      </c>
-      <c r="F24" s="1">
-        <f>F21-F8*10%+F13</f>
-        <v>160</v>
-      </c>
-      <c r="G24" s="7">
-        <f>G21-G8*10%+G13</f>
-        <v>1890</v>
-      </c>
-      <c r="H24" s="1">
-        <f>H21-H8*10%+H13</f>
-        <v>1190</v>
+      <c r="L23">
+        <f>L19+L22</f>
+        <v>8100</v>
       </c>
     </row>
     <row r="25" spans="4:12">
       <c r="D25" t="s">
         <v>27</v>
       </c>
-      <c r="E25" s="9">
-        <f>E24/E8</f>
+      <c r="E25" s="10">
+        <f>E22-E8*10%+E14</f>
+        <v>500</v>
+      </c>
+      <c r="F25" s="2">
+        <f>F22-F8*10%+F14</f>
+        <v>160</v>
+      </c>
+      <c r="G25" s="10">
+        <f>G22-G8*10%+G14</f>
+        <v>1890</v>
+      </c>
+      <c r="H25" s="2">
+        <f>H22-H8*10%+H14</f>
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="26" spans="4:12">
+      <c r="D26" t="s">
+        <v>28</v>
+      </c>
+      <c r="E26" s="12">
+        <f>E25/E8</f>
         <v>0.625</v>
       </c>
-      <c r="F25" s="10">
-        <f>F24/F8</f>
+      <c r="F26" s="13">
+        <f>F25/F8</f>
         <v>0.4</v>
       </c>
-      <c r="G25" s="9">
-        <f>G24/G8</f>
+      <c r="G26" s="12">
+        <f>G25/G8</f>
         <v>0.525</v>
       </c>
-      <c r="H25" s="10">
-        <f>H24/H8</f>
-        <v>0.330555555555556</v>
-      </c>
-    </row>
-    <row r="27" spans="4:12">
-      <c r="D27" t="s">
-        <v>28</v>
+      <c r="H26" s="13">
+        <f>H25/H8</f>
+        <v>0.280555555555556</v>
+      </c>
+    </row>
+    <row r="28" spans="4:12">
+      <c r="D28" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1818,107 +1839,106 @@
   <sheetData>
     <row r="4" spans="2:6">
       <c r="C4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" s="1" customFormat="1" spans="2:6">
-      <c r="C6" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="1" t="s">
+    </row>
+    <row r="6" s="2" customFormat="1" spans="2:6">
+      <c r="C6" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="D6" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="E6" s="2" t="s">
         <v>33</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="2:6">
       <c r="C7">
-        <v>3500</v>
-      </c>
-      <c r="D7" s="2">
-        <f>C7*12</f>
-        <v>42000</v>
-      </c>
-    </row>
-    <row r="8" s="2" customFormat="1" ht="39" customHeight="1" spans="2:6">
-      <c r="B8" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="3" t="s">
+        <v>3300</v>
+      </c>
+      <c r="D7" s="3">
+        <v>36000</v>
+      </c>
+    </row>
+    <row r="8" s="3" customFormat="1" ht="39" customHeight="1" spans="2:6">
+      <c r="B8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="C8" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="E8" s="6" t="s">
         <v>38</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="9" customFormat="1" ht="48" customHeight="1" spans="2:6">
       <c r="B9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" ht="63" customHeight="1" spans="2:6">
       <c r="B10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="C10" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="E10" s="2" t="s">
         <v>46</v>
       </c>
+      <c r="F10" s="2" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="11" spans="2:6">
-      <c r="E11" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F11" s="1" t="s">
+      <c r="E11" s="8" t="s">
         <v>48</v>
       </c>
+      <c r="F11" s="2" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="12" spans="2:6">
-      <c r="E12" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="F12" s="1" t="s">
+      <c r="E12" s="2" t="s">
         <v>50</v>
       </c>
+      <c r="F12" s="2" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="13" spans="2:6">
-      <c r="C13" s="4" t="s">
-        <v>51</v>
+      <c r="C13" s="9" t="s">
+        <v>52</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="2:6">
       <c r="C14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D14">
         <v>36000</v>
@@ -1926,10 +1946,43 @@
     </row>
     <row r="15" spans="2:6">
       <c r="C15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D15">
         <v>18000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="D4:F5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="4" outlineLevelCol="5"/>
+  <cols>
+    <col min="5" max="6" width="12.6875"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="4:6">
+      <c r="D4" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="4:6">
+      <c r="D5">
+        <v>200</v>
+      </c>
+      <c r="E5">
+        <f>82/91</f>
+        <v>0.901098901098901</v>
+      </c>
+      <c r="F5">
+        <f>D5*(1-E5)</f>
+        <v>19.7802197802198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: resolve PlatformAiTab build error & prevent duplicate brand creation on subscription
</commit_message>
<xml_diff>
--- a/amc_budgetaryplan.xlsx
+++ b/amc_budgetaryplan.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="10700"/>
+    <workbookView windowWidth="25600" windowHeight="10680"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1401,9 +1401,9 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="4" max="4" width="28.1875" customWidth="1"/>
-    <col min="5" max="5" width="12.6875" style="10"/>
+    <col min="5" max="5" width="15.359375" style="10" customWidth="1"/>
     <col min="6" max="6" width="14.625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="12.890625" style="10" customWidth="1"/>
+    <col min="7" max="7" width="12.109375" style="10" customWidth="1"/>
     <col min="8" max="8" width="12.6875" style="2"/>
     <col min="9" max="9" width="9" style="2"/>
     <col min="10" max="10" width="16.0625" style="10" customWidth="1"/>
@@ -1469,13 +1469,13 @@
         <v>800</v>
       </c>
       <c r="F8" s="2">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="G8" s="10">
         <v>3600</v>
       </c>
       <c r="H8" s="2">
-        <v>3600</v>
+        <v>3000</v>
       </c>
       <c r="I8" s="2">
         <v>3600</v>
@@ -1514,15 +1514,9 @@
       <c r="F10" s="2">
         <v>60</v>
       </c>
-      <c r="G10" s="10">
-        <v>500</v>
-      </c>
-      <c r="H10" s="2">
-        <v>180</v>
-      </c>
-      <c r="I10" s="2">
-        <v>2000</v>
-      </c>
+      <c r="G10" s="10"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
       <c r="J10" s="10" t="s">
         <v>12</v>
       </c>
@@ -1532,15 +1526,21 @@
       </c>
       <c r="L10">
         <f>H10*H6</f>
-        <v>1800</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="4:15">
       <c r="D11" t="s">
         <v>13</v>
       </c>
+      <c r="G11" s="10">
+        <v>800</v>
+      </c>
       <c r="H11" s="2">
-        <v>1200</v>
+        <v>800</v>
+      </c>
+      <c r="I11" s="2">
+        <v>2000</v>
       </c>
     </row>
     <row r="12" spans="4:15">
@@ -1553,6 +1553,12 @@
       <c r="F12" s="2">
         <v>20</v>
       </c>
+      <c r="G12" s="10">
+        <v>20</v>
+      </c>
+      <c r="H12" s="2">
+        <v>20</v>
+      </c>
       <c r="L12">
         <f>F12*F6*3</f>
         <v>3000</v>
@@ -1592,10 +1598,11 @@
       </c>
       <c r="F14" s="2">
         <f>F8*10%</f>
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="G14" s="10">
-        <v>200</v>
+        <f>G8*10%</f>
+        <v>360</v>
       </c>
       <c r="H14" s="2">
         <v>200</v>
@@ -1634,17 +1641,19 @@
       </c>
       <c r="F16" s="2">
         <f>F8*5%</f>
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G16" s="10">
-        <v>150</v>
+        <f>G8*5%</f>
+        <v>180</v>
       </c>
       <c r="H16" s="2">
+        <f>H8*5%</f>
         <v>150</v>
       </c>
       <c r="K16">
         <f>F6*F16</f>
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="L16">
         <f>H16*H6</f>
@@ -1681,7 +1690,7 @@
       </c>
       <c r="L19">
         <f>H6*H8*H19</f>
-        <v>1800</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="20" spans="4:12">
@@ -1711,18 +1720,18 @@
       </c>
       <c r="F22" s="2">
         <f>F8-SUM(F9:F16)</f>
-        <v>160</v>
+        <v>330</v>
       </c>
       <c r="G22" s="10">
         <f>G8-SUM(G9:G16)</f>
-        <v>2050</v>
+        <v>1540</v>
       </c>
       <c r="H22" s="2">
         <f>H8-SUM(H9:H16)</f>
-        <v>1170</v>
+        <v>1130</v>
       </c>
       <c r="I22" s="2">
-        <f>I8-I9-I10-I14-I13-I16</f>
+        <f>I8-I9-I11-I14-I13-I16</f>
         <v>1100</v>
       </c>
       <c r="J22" s="10" t="s">
@@ -1730,11 +1739,11 @@
       </c>
       <c r="K22">
         <f>K10+K16</f>
-        <v>4000</v>
+        <v>4500</v>
       </c>
       <c r="L22">
         <f>L10+L12+L16</f>
-        <v>6300</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="23" spans="4:12">
@@ -1747,26 +1756,26 @@
       </c>
       <c r="F23" s="13">
         <f>F22/F8</f>
-        <v>0.4</v>
+        <v>0.55</v>
       </c>
       <c r="G23" s="12">
         <f>G22/G8</f>
-        <v>0.569444444444444</v>
+        <v>0.427777777777778</v>
       </c>
       <c r="H23" s="13">
         <f>H22/H8</f>
-        <v>0.325</v>
+        <v>0.376666666666667</v>
       </c>
       <c r="J23" s="10" t="s">
         <v>26</v>
       </c>
       <c r="K23">
         <f>K19+K22</f>
-        <v>5200</v>
+        <v>5700</v>
       </c>
       <c r="L23">
         <f>L19+L22</f>
-        <v>8100</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="25" spans="4:12">
@@ -1779,15 +1788,15 @@
       </c>
       <c r="F25" s="2">
         <f>F22-F8*10%+F14</f>
-        <v>160</v>
+        <v>330</v>
       </c>
       <c r="G25" s="10">
         <f>G22-G8*10%+G14</f>
-        <v>1890</v>
+        <v>1540</v>
       </c>
       <c r="H25" s="2">
         <f>H22-H8*10%+H14</f>
-        <v>1010</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="26" spans="4:12">
@@ -1800,15 +1809,15 @@
       </c>
       <c r="F26" s="13">
         <f>F25/F8</f>
-        <v>0.4</v>
+        <v>0.55</v>
       </c>
       <c r="G26" s="12">
         <f>G25/G8</f>
-        <v>0.525</v>
+        <v>0.427777777777778</v>
       </c>
       <c r="H26" s="13">
         <f>H25/H8</f>
-        <v>0.280555555555556</v>
+        <v>0.343333333333333</v>
       </c>
     </row>
     <row r="28" spans="4:12">

</xml_diff>